<commit_message>
2026/06/07 Stage C-1 Kaggle 0–21 → FwuSow 0–31 reuse0_21_scaler 直接遷移，且沿用 0–21 尺度，測試外推
</commit_message>
<xml_diff>
--- a/notebook/DOE筆記.xlsx
+++ b/notebook/DOE筆記.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HoChePing\北科大_碩班_AI學程\期刊研究\使用LSTM模型預測福壽雞隻重量\Code程式碼\LSTM_TransferLearning_ChickWeight\notebook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648CF472-1BE0-4474-ADA1-AF574732161F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645A8689-9644-406D-B690-916E71CCB0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DOE－實驗設計" sheetId="6" r:id="rId1"/>
     <sheet name="DOE－拆解問題" sheetId="7" r:id="rId2"/>
     <sheet name="分階段實驗" sheetId="8" r:id="rId3"/>
     <sheet name="實驗步驟" sheetId="2" r:id="rId4"/>
-    <sheet name="正規化區分" sheetId="1" r:id="rId5"/>
-    <sheet name="Positive TL定義" sheetId="3" r:id="rId6"/>
-    <sheet name="Fwusow檔案說明" sheetId="4" r:id="rId7"/>
+    <sheet name="Stage C-2 和 Stage A、Stage C-1 的" sheetId="9" r:id="rId5"/>
+    <sheet name="正規化區分" sheetId="1" r:id="rId6"/>
+    <sheet name="Positive TL定義" sheetId="3" r:id="rId7"/>
+    <sheet name="Fwusow檔案說明" sheetId="4" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="110">
   <si>
     <t>資料版本</t>
   </si>
@@ -337,6 +338,33 @@
   </si>
   <si>
     <t>Stage C</t>
+  </si>
+  <si>
+    <t>任務</t>
+  </si>
+  <si>
+    <t>重點</t>
+  </si>
+  <si>
+    <t>日齡完全對齊，驗證 TL 是否有效</t>
+  </si>
+  <si>
+    <t>Stage C-1</t>
+  </si>
+  <si>
+    <t>Kaggle 0–21 → FwuSow 0–31 reuse0_21_scaler</t>
+  </si>
+  <si>
+    <t>直接遷移，且沿用 0–21 尺度，測試外推</t>
+  </si>
+  <si>
+    <t>Stage C-2</t>
+  </si>
+  <si>
+    <t>Kaggle 0–21 → FwuSow 0–31 fit0_31_full_scaler / own scaler</t>
+  </si>
+  <si>
+    <t>完整 0–31 Target task，測試 Source pre-train 是否仍有幫助</t>
   </si>
 </sst>
 </file>
@@ -861,7 +889,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="31.5">
+    <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
         <v>97</v>
       </c>
@@ -872,7 +900,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="63">
+    <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
         <v>98</v>
       </c>
@@ -883,7 +911,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="31.5">
+    <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
         <v>100</v>
       </c>
@@ -1026,6 +1054,64 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118ECCEC-5899-4501-8C65-FD443B516BE4}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="3" width="35.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="78.75">
+      <c r="A2" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="94.5">
+      <c r="A3" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="141.75">
+      <c r="A4" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
@@ -1073,7 +1159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73B2FDBF-13D3-44EC-B21D-0096BBE6BB69}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
@@ -1187,7 +1273,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AABAAA1C-57F3-4E3C-8B50-0B87A2146085}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15.75"/>

</xml_diff>

<commit_message>
2026/06/07 Stage C-1 Kaggle 0–21 → FwuSow 0–31 fit0_31_full_scaler 直接遷移，改用0-31 scaler 尺度，測試外推
</commit_message>
<xml_diff>
--- a/notebook/DOE筆記.xlsx
+++ b/notebook/DOE筆記.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HoChePing\北科大_碩班_AI學程\期刊研究\使用LSTM模型預測福壽雞隻重量\Code程式碼\LSTM_TransferLearning_ChickWeight\notebook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645A8689-9644-406D-B690-916E71CCB0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87D478E-444B-411C-BC92-5C9B666D43DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="119">
   <si>
     <t>資料版本</t>
   </si>
@@ -365,6 +365,33 @@
   </si>
   <si>
     <t>完整 0–31 Target task，測試 Source pre-train 是否仍有幫助</t>
+  </si>
+  <si>
+    <t>建議名稱</t>
+  </si>
+  <si>
+    <t>Scaler 設定</t>
+  </si>
+  <si>
+    <t>實驗定位</t>
+  </si>
+  <si>
+    <t>StageC-1_DirectTransfer_Kaggle0_21_to_FwuSow0_31_reuse0_21_scaler</t>
+  </si>
+  <si>
+    <t>沿用 FwuSow 0–21 scaler</t>
+  </si>
+  <si>
+    <t>與 Stage B 比較用，檢查直接遷移是否不如分階段遷移</t>
+  </si>
+  <si>
+    <t>StageC-2_DirectTransfer_Kaggle0_21_to_FwuSow0_31_fit0_31_full_scaler</t>
+  </si>
+  <si>
+    <t>使用 FwuSow 0–31 全區間 fit scaler</t>
+  </si>
+  <si>
+    <t>補充實驗，檢查完整 0–31 normalized scale 下直接遷移效果</t>
   </si>
 </sst>
 </file>
@@ -1055,13 +1082,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118ECCEC-5899-4501-8C65-FD443B516BE4}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="3" width="35.7109375" customWidth="1"/>
+    <col min="1" max="4" width="35.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -1072,7 +1099,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="78.75">
+    <row r="2" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>97</v>
       </c>
@@ -1083,7 +1110,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="94.5">
+    <row r="3" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>104</v>
       </c>
@@ -1094,7 +1121,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="141.75">
+    <row r="4" spans="1:4" ht="39.950000000000003" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>107</v>
       </c>
@@ -1103,6 +1130,48 @@
       </c>
       <c r="C4" s="4" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="31.5">
+      <c r="A8" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="126">
+      <c r="A9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="126">
+      <c r="A10" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>